<commit_message>
Add bootstrap decisions and build dataset scripts for family office intelligence
- Introduced `bootstrap_decisions.py` to convert family office records from JSON to a structured decision format.
- Added `build_dataset.py` to enrich family office data using SEC and ProPublica APIs, enhancing the dataset with live data retrieval.
- Created `decisions.json` to store processed decisions for further analysis.
- Updated `family_offices.json` with new fields for pipeline provenance and adjusted existing data for consistency.
- Added `VALIDATION_CHAINS.md` to document the validation process for family office records, ensuring transparency in data handling.
- Updated `README.md` with the new live demo link for better accessibility.
</commit_message>
<xml_diff>
--- a/family_offices_export.xlsx
+++ b/family_offices_export.xlsx
@@ -658,7 +658,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Duquesne Family Office LLC is a single-family office in New York, NY, serving the Druckenmiller family (founded 2010). Investment focus: concentrated global macro; multi-asset across public and private markets. Estimated AUM: $4B-$8B. Key decision-makers: Stanley Druckenmiller (Founder / Chairman). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Duquesne Family Office LLC is a single-family office in NEW YORK, NY, serving the Druckenmiller family (founded 2010). Investment focus: concentrated global macro; multi-asset across public and private markets. Estimated AUM: $4B-$8B. Key decision-makers: Stanley Druckenmiller (Founder / Chairman). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -678,7 +678,7 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>NEW YORK</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>The Jeffrey Company (Jeffrey Fiduciary Co.) is a single-family office in Columbus, OH, serving the Jeffrey family (~9 staff). Investment focus: global investment fund, family office and trust services; long-horizon multi-asset. AUM not publicly disclosed. Key decision-makers: Kerry Houghton (CEO). Firm contact: phone (614) 221-6115; email info@jeffreyfc.com; website jeffreyco.com; 140 East Town Street, Suite 1400, Columbus, OH 43215. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>The Jeffrey Company (Jeffrey Fiduciary Co.) is a single-family office in COLUMBUS, OH, serving the Jeffrey family. Investment focus: global investment fund, family office and trust services; long-horizon multi-asset. AUM not publicly disclosed. Key decision-makers: Kerry Houghton (CEO). Firm contact: phone (614) 221-6115; email info@jeffreyfc.com; website jeffreyco.com; 140 East Town Street, Suite 1400, Columbus, OH 43215. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>COLUMBUS</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Henry Crown and Company (HCC) is a single-family office in Chicago, IL, serving the Crown family (founded 1959, ~200 professionals). Investment focus: public securities, real estate, private equity, infrastructure, operating companies, sports franchises (Bulls; Aspen Skiing; Alterra). AUM not publicly disclosed. Key decision-makers: Steve Crown (Executive Chairman); Bill Crown (President &amp; CEO). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Henry Crown and Company (HCC) is a single-family office in Chicago, IL, serving the Crown family (founded 1959). Investment focus: public securities, real estate, private equity, infrastructure, operating companies, sports franchises (Bulls; Aspen Skiing; Alterra). AUM not publicly disclosed. Key decision-makers: Steve Crown (Executive Chairman); Bill Crown (President &amp; CEO). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>The Sobrato Organization (TSO) is a single-family office in Mountain View, CA, serving the Sobrato family (founded 1979, ~70-95 staff). Investment focus: commercial real estate (office/R&amp;D), multifamily communities, and long-horizon direct investing via Sobrato Capital; no outside equity partners. AUM not disclosed; portfolio ~7.5M sq ft office/R&amp;D + ~7,500 multifamily units. Key decision-makers: John A. Sobrato (Founder &amp; Chairman); John Michael Sobrato (Family Principal); Tony Mestres (CEO). Firm contact: website sobrato.com. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>The Sobrato Organization (TSO) is a single-family office in Mountain View, CA, serving the Sobrato family (founded 1979). Investment focus: commercial real estate (office/R&amp;D), multifamily communities, and long-horizon direct investing via Sobrato Capital; no outside equity partners. AUM not disclosed; portfolio ~7.5M sq ft office/R&amp;D + ~7,500 multifamily units. Key decision-makers: John A. Sobrato (Founder &amp; Chairman); John Michael Sobrato (Family Principal); Tony Mestres (CEO). Firm contact: website sobrato.com. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Karsh Family Office is a single-family office in Los Angeles, CA, serving the Karsh family. Investment focus: private/alternative market investments and venture co-investments; large-scale philanthropy (higher ed, civic education). AUM not disclosed. Key decision-makers: Bruce Karsh (Principal (co-founder/CIO of Oaktree Capital)); Martha Karsh (Principal). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Karsh Family Office is a single-family office in Beverly Hills, CA, serving the Karsh family. Investment focus: private/alternative market investments and venture co-investments; large-scale philanthropy (higher ed, civic education). Estimated AUM: ~$336M. Key decision-makers: Bruce Karsh (Principal (co-founder/CIO of Oaktree Capital)); Martha Karsh (Principal). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1129,7 +1129,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Beverly Hills</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Hall Family Foundation is a single-family office in Kansas City, MO, serving the Hall family. Investment focus: Greater Kansas City philanthropy — community quality of life, systemic solutions to community needs, education and civic initiatives. Estimated AUM: ~$1.03B. Firm contact: website hallfamilyfoundation.org.</t>
+          <t>Hall Family Foundation is a single-family office in Kansas City, MO, serving the Hall family. Investment focus: Greater Kansas City philanthropy — community quality of life, systemic solutions to community needs, education and civic initiatives. Estimated AUM: ~$1.0B. Firm contact: website hallfamilyfoundation.org.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Poses Family Foundation is a single-family office in Florham Park, NJ, serving the Poses family (founded 2004). Investment focus: learning and thinking differences (learning disabilities), K-12 education, human services, mental health, and the arts; combines grants with operational capacity-building. Estimated AUM: ~$730M. Key decision-makers: Nancy Poses (Co-Founder); Fred Poses (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Poses Family Foundation is a single-family office in Florham Park, NJ, serving the Poses family (founded 2004). Investment focus: learning and thinking differences (learning disabilities), K-12 education, human services, mental health, and the arts; combines grants with operational capacity-building. Estimated AUM: ~$630M. Key decision-makers: Nancy Poses (Co-Founder); Fred Poses (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Stanley Family Foundation is a single-family office in Briarcliff Manor, NY, serving the Stanley family (founded 1985). Investment focus: psychiatric research — concentrated, invitation-only giving to human genetics, neurobiology, and computational research on schizophrenia and bipolar disorder, chiefly via the Stanley Center at the Broad Institute. Estimated AUM: ~$554M.</t>
+          <t>Stanley Family Foundation is a single-family office in Briarcliff, NY, serving the Stanley family (founded 1985). Investment focus: psychiatric research — concentrated, invitation-only giving to human genetics, neurobiology, and computational research on schizophrenia and bipolar disorder, chiefly via the Stanley Center at the Broad Institute. Estimated AUM: ~$554M.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1457,7 +1457,7 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Briarcliff Manor</t>
+          <t>Briarcliff</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -2035,14 +2035,14 @@
         <v>2026</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Pathy Family Foundation is a single-family office in Montreal, QC, serving the Pathy family. Investment focus: advancing dignity, rights, and empowerment of communities in Canada and globally; genuine partnership, collaboration, and support for community-led social change. Estimated AUM: ~$247M.</t>
+          <t>Pathy Family Foundation is a single-family office in Canada, None, serving the Pathy family. Investment focus: advancing dignity, rights, and empowerment of communities in Canada and globally; genuine partnership, collaboration, and support for community-led social change. Estimated AUM: ~$247M.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2062,14 +2062,10 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Montreal</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>QC</t>
-        </is>
-      </c>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
           <t>Canada</t>
@@ -2109,7 +2105,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Edgerley Family Foundation is a single-family office in Boston, MA, serving the Edgerley family (founded 2004). Investment focus: education and leadership, youth opportunity, community health, and homeless/social services, focused on Massachusetts and New England; relationship-driven, no public applications. Estimated AUM: ~$239M. Key decision-makers: Paul Edgerley (Co-Founder); Sandra Edgerley (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Edgerley Family Foundation is a single-family office in Overland Park, KS, serving the Edgerley family (founded 2004). Investment focus: education and leadership, youth opportunity, community health, and homeless/social services, focused on Massachusetts and New England; relationship-driven, no public applications. Estimated AUM: ~$225M. Key decision-makers: Paul Edgerley (Co-Founder); Sandra Edgerley (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2129,12 +2125,12 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Overland Park</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2192,7 +2188,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Hao Family Foundation is a single-family office in Saratoga Springs, NY, serving the Hao family (founded 2017). Investment focus: impact-oriented grantmaking; funding directed toward community and impact investment portfolios (e.g., Turner Impact Capital). Estimated AUM: ~$188M-$304M.</t>
+          <t>Hao Family Foundation is a single-family office in Saratoga Spgs, NY, serving the Hao family (founded 2017). Investment focus: impact-oriented grantmaking; funding directed toward community and impact investment portfolios (e.g., Turner Impact Capital). Estimated AUM: ~$188M.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2212,7 +2208,7 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Saratoga Springs</t>
+          <t>Saratoga Spgs</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2500,7 +2496,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Bezos Expeditions is a single-family office in Mercer Island, WA, serving the Bezos family (founded 2005, ~150+ staff). Investment focus: venture capital, private equity, and direct personal investments — disruptive technology, aerospace (Blue Origin), and media (The Washington Post). Estimated AUM: ~$100B-$200B. Key decision-makers: Melinda Lewison (Managing Director); Jeff Bezos (Principal). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Bezos Expeditions is a single-family office in Mercer Island, WA, serving the Bezos family (founded 2005). Investment focus: venture capital, private equity, and direct personal investments — disruptive technology, aerospace (Blue Origin), and media (The Washington Post). Estimated AUM: ~$100B-$200B. Key decision-makers: Melinda Lewison (Managing Director); Jeff Bezos (Principal). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2583,7 +2579,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Linde Family Foundation is a single-family office in Boston, MA, serving the Linde family (founded 2000). Investment focus: arts, education, youth/children's services, and medical research in greater Boston (Dana-Farber, Tanglewood, MFA, Beth Israel Deaconess); no public application process. Estimated AUM: ~$214M. Key decision-makers: Joyce Linde (Co-Founder / Trustee). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Linde Family Foundation is a single-family office in Boston, MA, serving the Linde family (founded 2000). Investment focus: arts, education, youth/children's services, and medical research in greater Boston (Dana-Farber, Tanglewood, MFA, Beth Israel Deaconess); no public application process. Estimated AUM: ~$160M. Key decision-makers: Joyce Linde (Co-Founder / Trustee). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2749,7 +2745,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Sundheim Family Foundation is a single-family office in New York, NY, serving the Sundheim family. Investment focus: higher-education student aid, medical research (type 1 diabetes), and contemporary art; major gifts to UPenn and the Diabetes Research Institute. Estimated AUM: ~$104M. Key decision-makers: Daniel Sundheim (Co-Founder); Brett Sundheim (Co-Founder). Firm contact: C/O Sunny Cap Management, 9 W 57th St, New York, NY. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Sundheim Family Foundation is a single-family office in New York, NY, serving the Sundheim family. Investment focus: higher-education student aid, medical research (type 1 diabetes), and contemporary art; major gifts to UPenn and the Diabetes Research Institute. Estimated AUM: ~$83M. Key decision-makers: Daniel Sundheim (Co-Founder); Brett Sundheim (Co-Founder). Firm contact: C/O Sunny Cap Management, 9 W 57th St, New York, NY. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2896,14 +2892,14 @@
         <v>2026</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Tsao Foundation is a single-family office in Singapore, None, serving the Tsao family. Investment focus: enhancing quality of life for older persons; community-based eldercare, health and social services (Hua Mei), ageing-in-place and self-determination for seniors. Estimated AUM: ~$88M. Key decision-makers: Dr Mary Ann Tsao (Chairman / Founding Director). Firm contact: website tsaofoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Tsao Foundation is a single-family office in Corona Dl Mar, CA, serving the Tsao family. Investment focus: enhancing quality of life for older persons; community-based eldercare, health and social services (Hua Mei), ageing-in-place and self-determination for seniors. Estimated AUM: ~$88M. Key decision-makers: Dr Mary Ann Tsao (Chairman / Founding Director). Firm contact: website tsaofoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2935,10 +2931,14 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr"/>
+          <t>Corona Dl Mar</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
           <t>Singapore</t>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Crabill Family Foundation is a single-family office in San Francisco, CA, serving the Crabill family (founded 2018). Investment focus: access to healthcare, education, housing, and arts, focused on Springfield, OH and San Francisco, CA; strategy still developing. Estimated AUM: ~$54M. Key decision-makers: Scott Crabill (Co-Founder); Angela Crabill (Co-Founder). Firm contact: email hello@crabillfamilyfoundation.org; website crabillfamilyfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Crabill Family Foundation is a single-family office in Denver, CO, serving the Crabill family (founded 2018). Investment focus: access to healthcare, education, housing, and arts, focused on Springfield, OH and San Francisco, CA; strategy still developing. Estimated AUM: ~$12M. Key decision-makers: Scott Crabill (Co-Founder); Angela Crabill (Co-Founder). Firm contact: email hello@crabillfamilyfoundation.org; website crabillfamilyfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3196,12 +3196,12 @@
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Spaht Family Foundation is a single-family office in San Francisco, CA, serving the Spaht family (founded 2019). Investment focus: climate, mental health, and the arts; long-term US impact via grants and field-building (e.g., Lindley Center for Student Wellness at W&amp;L; SMU Meadows School of the Arts). Estimated AUM: ~$49.7M. Key decision-makers: Holden Spaht (Co-Founder); Claire Spaht (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Spaht Family Foundation is a single-family office in San Francisco, CA, serving the Spaht family (founded 2019). Investment focus: climate, mental health, and the arts; long-term US impact via grants and field-building (e.g., Lindley Center for Student Wellness at W&amp;L; SMU Meadows School of the Arts). Estimated AUM: ~$50M. Key decision-makers: Holden Spaht (Co-Founder); Claire Spaht (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Towle Family Foundation is a single-family office in Greenwood Village, CO, serving the Towle family. Investment focus: endowments, scholarships, and educational/community outreach; relationship-driven, no public application process. Estimated AUM: ~$42M. Key decision-makers: Christopher D. Towle (Officer); Perry E. Towle (Officer). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Towle Family Foundation is a single-family office in Greenwood Vlg, CO, serving the Towle family. Investment focus: endowments, scholarships, and educational/community outreach; relationship-driven, no public application process. Estimated AUM: ~$42M. Key decision-makers: Christopher D. Towle (Officer); Perry E. Towle (Officer). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3457,7 +3457,7 @@
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Greenwood Village</t>
+          <t>Greenwood Vlg</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Yarbrough Family Foundation is a single-family office in Franklin, TN, serving the Yarbrough family (founded 2007). Investment focus: education and youth (Battle Ground Academy), health and human services, and Christian/community outreach. Estimated AUM: ~$24M. Key decision-makers: Jon Yarbrough (Founder). Firm contact: phone (615) 538-5636. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Yarbrough Family Foundation is a single-family office in Franklin, TN, serving the Yarbrough family (founded 2007). Investment focus: education and youth (Battle Ground Academy), health and human services, and Christian/community outreach. Estimated AUM: ~$28M. Key decision-makers: Jon Yarbrough (Founder). Firm contact: phone (615) 538-5636. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Baustert Family Foundation is a single-family office in St. Paul, MN, serving the Baustert family (founded 2016). Investment focus: education, health sciences, and human services in Illinois and Minnesota; invitation-only, family-run board (e.g., $40M gift to NIU's Baustert Bahwell Health Technology Center). Estimated AUM: ~$78M. Key decision-makers: James Baustert (Co-Founder); Theo Baustert (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Baustert Family Foundation is a single-family office in St Paul, MN, serving the Baustert family (founded 2016). Investment focus: education, health sciences, and human services in Illinois and Minnesota; invitation-only, family-run board (e.g., $40M gift to NIU's Baustert Bahwell Health Technology Center). Estimated AUM: ~$31M. Key decision-makers: James Baustert (Co-Founder); Theo Baustert (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3801,7 +3801,7 @@
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>St. Paul</t>
+          <t>St Paul</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Mondre Family Foundation is a single-family office in New York, NY, serving the Mondre family (founded 2019). Investment focus: educational access and middle-income student financial aid (e.g., $20M Mondre Family Initiative at UPenn). Estimated AUM: ~$51M. Key decision-makers: Greg Mondre (Co-Founder); Alexandra Mondre (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Mondre Family Foundation is a single-family office in New York, NY, serving the Mondre family (founded 2019). Investment focus: educational access and middle-income student financial aid (e.g., $20M Mondre Family Initiative at UPenn). Estimated AUM: ~$16M. Key decision-makers: Greg Mondre (Co-Founder); Alexandra Mondre (Co-Founder). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Konzen Family Foundation is a single-family office in Bellevue, WA, serving the Konzen family. Investment focus: grantmaking to pre-selected charitable groups (e.g., CARE USA) and community organizations; invitation-only, trustee-selected. Estimated AUM: ~$18M.</t>
+          <t>Konzen Family Foundation is a single-family office in Issaquah, WA, serving the Konzen family. Investment focus: grantmaking to pre-selected charitable groups (e.g., CARE USA) and community organizations; invitation-only, trustee-selected. Estimated AUM: ~$18M.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3967,7 +3967,7 @@
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>Issaquah</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Dunlap Family Foundation is a single-family office in Canonsburg, PA, serving the Dunlap family. Investment focus: faith-inspired giving for human services, education, and strengthening families in the Greater Pittsburgh region. Estimated AUM: ~$64M. Key decision-makers: Edward B. Dunlap Jr. (Namesake / Family Principal). Firm contact: email privatefoundationsolutions@pnc.com. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Dunlap Family Foundation is a single-family office in Canonsburg, PA, serving the Dunlap family. Investment focus: faith-inspired giving for human services, education, and strengthening families in the Greater Pittsburgh region. Estimated AUM: ~$0M. Key decision-makers: Edward B. Dunlap Jr. (Namesake / Family Principal). Firm contact: email privatefoundationsolutions@pnc.com. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Adelson Family Foundation is a single-family office in Needham, MA, serving the Adelson family (founded 2007). Investment focus: strengthening Israel and the Jewish people — Israel advocacy, Jewish/Zionist education (Birthright), Holocaust and antisemitism awareness, and welfare/healthcare. AUM 990 assets modest (~$743K); operates as a flow-through funding tens of millions annually. Key decision-makers: Dr. Miriam Adelson (Chair / Principal). Firm contact: website adelsonfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Adelson Family Foundation is a single-family office in Needham, MA, serving the Adelson family (founded 2007). Investment focus: strengthening Israel and the Jewish people — Israel advocacy, Jewish/Zionist education (Birthright), Holocaust and antisemitism awareness, and welfare/healthcare. Estimated AUM: ~$1M. Key decision-makers: Dr. Miriam Adelson (Chair / Principal). Firm contact: website adelsonfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Kopp Family Office, LLC is a single-family office in Minnetonka, MN, serving the Kopp family. Investment focus: manages the Kopp family's private wealth and public-equity portfolio (ETFs and major equities); related family philanthropy in education and emergency assistance in Minnesota. Estimated AUM: ~$163M. Key decision-makers: Kopp family (Lee Kopp legacy) (Principals). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Kopp Family Office, LLC is a single-family office in MINNETONKA, MN, serving the Kopp family. Investment focus: manages the Kopp family's private wealth and public-equity portfolio (ETFs and major equities); related family philanthropy in education and emergency assistance in Minnesota. Estimated AUM: ~$163M. Key decision-makers: Kopp family (Lee Kopp legacy) (Principals). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4378,7 +4378,7 @@
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Minnetonka</t>
+          <t>MINNETONKA</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Kallir Family Foundation is a single-family office in New York, NY, serving the Kallir family. Investment focus: private family grantmaking foundation based in New York, NY. Estimated AUM: ~$51M. Key decision-makers: Jane Kallir (President). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Kallir Family Foundation is a single-family office in New York, NY, serving the Kallir family. Investment focus: private family grantmaking foundation based in New York, NY. Estimated AUM: ~$6M. Key decision-makers: Jane Kallir (President). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Winiarski Family Foundation is a single-family office in Napa, CA, serving the Winiarski family (founded 2007). Investment focus: education, conservation (Napa land/agricultural easements), healthcare, and preserving food and wine history; pre-selected partnerships, no unsolicited proposals. Estimated AUM: ~$14M. Key decision-makers: Barbara Winiarski (Co-Founder / Trustee). Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Winiarski Family Foundation is a single-family office in Yountville, CA, serving the Winiarski family (founded 2007). Investment focus: education, conservation (Napa land/agricultural easements), healthcare, and preserving food and wine history; pre-selected partnerships, no unsolicited proposals. Estimated AUM: ~$14M. Key decision-makers: Barbara Winiarski (Co-Founder / Trustee). Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -4544,7 +4544,7 @@
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Napa</t>
+          <t>Yountville</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Davis Family Foundation is a single-family office in Falmouth, ME, serving the Davis family (founded 1986). Investment focus: supporting educational, medical, and cultural/arts organizations primarily in Maine. AUM grantmaking foundation; net assets per 990. Key decision-makers: Phyllis C. Davis (Co-Founder); H. Halsey Davis (Co-Founder). Firm contact: website davisfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
+          <t>Davis Family Foundation is a single-family office in Hanover, MD, serving the Davis family (founded 1986). Investment focus: supporting educational, medical, and cultural/arts organizations primarily in Maine. Estimated AUM: ~$1.4B. Key decision-makers: Phyllis C. Davis (Co-Founder); H. Halsey Davis (Co-Founder). Firm contact: website davisfoundation.org. Direct contact details for individual decision-makers are not publicly available.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -4813,12 +4813,12 @@
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Falmouth</t>
+          <t>Hanover</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">

</xml_diff>